<commit_message>
Beispielskript zum Erstellen, Protokollieren und Verteilen aller Berichte
</commit_message>
<xml_diff>
--- a/daten/kohorte_berichte.xlsx
+++ b/daten/kohorte_berichte.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -380,6 +380,11 @@
           <t>Titel</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Ordner</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -434,6 +439,11 @@
           <t>Befragung 2025: Gesamtbericht</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Gesamtberichte | Musterwissenschaft | Beispielkunde</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -461,6 +471,11 @@
           <t>Befragung 2025: B.Sc. Musterwissenschaft</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Musterwissenschaft</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -488,6 +503,11 @@
           <t>Befragung 2025: M.Sc. Musterwissenschaft</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Musterwissenschaft</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -513,6 +533,11 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>Befragung 2025: B.A. Beispielkunde</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Beispielkunde</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Schrift mitgeliefert, Vorbereitungsskript mit fiktivem evasys-Export
</commit_message>
<xml_diff>
--- a/daten/kohorte_berichte.xlsx
+++ b/daten/kohorte_berichte.xlsx
@@ -409,7 +409,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Befragung 2025: Master-Bericht (alle Fragen)</t>
+          <t>Master-Bericht (alle Fragen)</t>
         </is>
       </c>
     </row>
@@ -436,7 +436,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Befragung 2025: Gesamtbericht</t>
+          <t>Gesamtbericht</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -468,7 +468,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Befragung 2025: B.Sc. Musterwissenschaft</t>
+          <t>B.Sc. Musterwissenschaft</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Befragung 2025: M.Sc. Musterwissenschaft</t>
+          <t>M.Sc. Musterwissenschaft</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -532,7 +532,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Befragung 2025: B.A. Beispielkunde</t>
+          <t>B.A. Beispielkunde</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Befragung 2025: Sonderauswertung</t>
+          <t>Sonderauswertung</t>
         </is>
       </c>
     </row>

</xml_diff>